<commit_message>
Ajusta auxiliares normalizados e marcadores da proposta
</commit_message>
<xml_diff>
--- a/dados/auxiliares.xlsx
+++ b/dados/auxiliares.xlsx
@@ -8,15 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://factofundacao-my.sharepoint.com/personal/katarina_lemos_facto_org_br/Documents/Área de Trabalho/my_codes/precificacao_doa/dados/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="9" documentId="8_{F0DCD92E-0CA8-4F9A-B9FD-597F54C575EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F3FE9D8-E659-450D-A581-BFF4F8F0A420}"/>
+  <xr:revisionPtr revIDLastSave="48" documentId="8_{F0DCD92E-0CA8-4F9A-B9FD-597F54C575EF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{4F95F20A-AA2F-4009-B4EA-46852C6B77E0}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="812" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="812" activeTab="6" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="CLASSIFICAÇÃO DE BOLSAS" sheetId="25" r:id="rId1"/>
-    <sheet name="CLASSIFICAÇÃO DE DESPESAS" sheetId="26" r:id="rId2"/>
-    <sheet name="CLASSIFICAÇÃO E VALORES DE DIÁR" sheetId="27" r:id="rId3"/>
-    <sheet name="CLASSIFICAÇÃO PASSAGENS " sheetId="29" r:id="rId4"/>
+    <sheet name="aux_bolsas" sheetId="30" r:id="rId2"/>
+    <sheet name="CLASSIFICAÇÃO DE DESPESAS" sheetId="26" r:id="rId3"/>
+    <sheet name="aux_despesas" sheetId="31" r:id="rId4"/>
+    <sheet name="CLASSIFICAÇÃO E VALORES DE DIÁR" sheetId="27" r:id="rId5"/>
+    <sheet name="aux_diarias" sheetId="32" r:id="rId6"/>
+    <sheet name="aux_passagem" sheetId="33" r:id="rId7"/>
+    <sheet name="CLASSIFICAÇÃO PASSAGENS " sheetId="29" r:id="rId8"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -39,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="513" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="374">
   <si>
     <t>Categoria</t>
   </si>
@@ -567,9 +571,6 @@
   </si>
   <si>
     <t>Intercambista Profissional - Qualificação/Experiente - INT-PQE</t>
-  </si>
-  <si>
-    <t>EQUIPAMENTOS E MATERIAIS PERMANENTES</t>
   </si>
   <si>
     <t>MATERIAL DE CONSUMO</t>
@@ -1132,6 +1133,39 @@
   <si>
     <t>Teto fator multiplicador</t>
   </si>
+  <si>
+    <t>MATERIAIS PERMANENTES</t>
+  </si>
+  <si>
+    <t>modalidade</t>
+  </si>
+  <si>
+    <t>categoria</t>
+  </si>
+  <si>
+    <t>valor_referencia</t>
+  </si>
+  <si>
+    <t>Material permanente</t>
+  </si>
+  <si>
+    <t>grupo_parf</t>
+  </si>
+  <si>
+    <t>Material de consumo</t>
+  </si>
+  <si>
+    <t>Serviço PJ</t>
+  </si>
+  <si>
+    <t>tipo_diaria</t>
+  </si>
+  <si>
+    <t>valor_unitario</t>
+  </si>
+  <si>
+    <t>tipo_passagem</t>
+  </si>
 </sst>
 </file>
 
@@ -1527,10 +1561,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{E1A5BAD7-D881-4D1D-9710-E0EA2711E2F8}" name="tCategorias" displayName="tCategorias" ref="A1:O41" totalsRowShown="0">
   <autoFilter ref="A1:O41" xr:uid="{E1A5BAD7-D881-4D1D-9710-E0EA2711E2F8}"/>
@@ -1892,7 +1922,7 @@
         <v>14</v>
       </c>
       <c r="H1" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="I1" s="2" t="s">
         <v>15</v>
@@ -3931,6 +3961,472 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{770B2F8B-B1BA-46C2-8829-3DBB78030F14}">
+  <dimension ref="A1:C41"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="66.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="74.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" t="s">
+        <v>364</v>
+      </c>
+      <c r="B1" t="s">
+        <v>365</v>
+      </c>
+      <c r="C1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3">
+      <c r="A2" t="s">
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3">
+      <c r="A3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="C3">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3">
+      <c r="A4" t="s">
+        <v>34</v>
+      </c>
+      <c r="B4" t="s">
+        <v>36</v>
+      </c>
+      <c r="C4">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3">
+      <c r="A5" t="s">
+        <v>38</v>
+      </c>
+      <c r="B5" t="s">
+        <v>40</v>
+      </c>
+      <c r="C5">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>42</v>
+      </c>
+      <c r="B6" t="s">
+        <v>44</v>
+      </c>
+      <c r="C6">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3">
+      <c r="A7" t="s">
+        <v>45</v>
+      </c>
+      <c r="B7" t="s">
+        <v>47</v>
+      </c>
+      <c r="C7">
+        <v>1100</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3">
+      <c r="A8" t="s">
+        <v>48</v>
+      </c>
+      <c r="B8" t="s">
+        <v>50</v>
+      </c>
+      <c r="C8">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>54</v>
+      </c>
+      <c r="B9" t="s">
+        <v>56</v>
+      </c>
+      <c r="C9">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3">
+      <c r="A10" t="s">
+        <v>57</v>
+      </c>
+      <c r="B10" t="s">
+        <v>59</v>
+      </c>
+      <c r="C10">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3">
+      <c r="A11" t="s">
+        <v>60</v>
+      </c>
+      <c r="B11" t="s">
+        <v>62</v>
+      </c>
+      <c r="C11">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3">
+      <c r="A12" t="s">
+        <v>63</v>
+      </c>
+      <c r="B12" t="s">
+        <v>65</v>
+      </c>
+      <c r="C12">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3">
+      <c r="A13" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" t="s">
+        <v>68</v>
+      </c>
+      <c r="C13">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3">
+      <c r="A14" t="s">
+        <v>69</v>
+      </c>
+      <c r="B14" t="s">
+        <v>71</v>
+      </c>
+      <c r="C14">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3">
+      <c r="A15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B15" t="s">
+        <v>74</v>
+      </c>
+      <c r="C15">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3">
+      <c r="A16" t="s">
+        <v>75</v>
+      </c>
+      <c r="B16" t="s">
+        <v>77</v>
+      </c>
+      <c r="C16">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17" t="s">
+        <v>78</v>
+      </c>
+      <c r="B17" t="s">
+        <v>80</v>
+      </c>
+      <c r="C17">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="A18" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s">
+        <v>6</v>
+      </c>
+      <c r="C18">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3">
+      <c r="A19" t="s">
+        <v>83</v>
+      </c>
+      <c r="B19" t="s">
+        <v>85</v>
+      </c>
+      <c r="C19">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3">
+      <c r="A20" t="s">
+        <v>86</v>
+      </c>
+      <c r="B20" t="s">
+        <v>88</v>
+      </c>
+      <c r="C20">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3">
+      <c r="A21" t="s">
+        <v>89</v>
+      </c>
+      <c r="B21" t="s">
+        <v>91</v>
+      </c>
+      <c r="C21">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3">
+      <c r="A22" t="s">
+        <v>92</v>
+      </c>
+      <c r="B22" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22">
+        <v>1500</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3">
+      <c r="A23" t="s">
+        <v>94</v>
+      </c>
+      <c r="B23" t="s">
+        <v>5</v>
+      </c>
+      <c r="C23">
+        <v>1400</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3">
+      <c r="A24" t="s">
+        <v>96</v>
+      </c>
+      <c r="B24" t="s">
+        <v>1</v>
+      </c>
+      <c r="C24">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3">
+      <c r="A25" t="s">
+        <v>98</v>
+      </c>
+      <c r="B25" t="s">
+        <v>7</v>
+      </c>
+      <c r="C25">
+        <v>1200</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3">
+      <c r="A26" t="s">
+        <v>100</v>
+      </c>
+      <c r="B26" t="s">
+        <v>3</v>
+      </c>
+      <c r="C26">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3">
+      <c r="A27" t="s">
+        <v>102</v>
+      </c>
+      <c r="B27" t="s">
+        <v>4</v>
+      </c>
+      <c r="C27">
+        <v>1300</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>104</v>
+      </c>
+      <c r="B28" t="s">
+        <v>106</v>
+      </c>
+      <c r="C28">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>110</v>
+      </c>
+      <c r="B29" t="s">
+        <v>112</v>
+      </c>
+      <c r="C29">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>116</v>
+      </c>
+      <c r="B30" t="s">
+        <v>118</v>
+      </c>
+      <c r="C30">
+        <v>2100</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3">
+      <c r="A31" t="s">
+        <v>119</v>
+      </c>
+      <c r="B31" t="s">
+        <v>121</v>
+      </c>
+      <c r="C31">
+        <v>700</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3">
+      <c r="A32" t="s">
+        <v>125</v>
+      </c>
+      <c r="B32" t="s">
+        <v>127</v>
+      </c>
+      <c r="C32">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3">
+      <c r="A33" t="s">
+        <v>131</v>
+      </c>
+      <c r="B33" t="s">
+        <v>133</v>
+      </c>
+      <c r="C33">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3">
+      <c r="A34" t="s">
+        <v>134</v>
+      </c>
+      <c r="B34" t="s">
+        <v>8</v>
+      </c>
+      <c r="C34">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3">
+      <c r="A35" t="s">
+        <v>136</v>
+      </c>
+      <c r="B35" t="s">
+        <v>138</v>
+      </c>
+      <c r="C35">
+        <v>3100</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3">
+      <c r="A36" t="s">
+        <v>142</v>
+      </c>
+      <c r="B36" t="s">
+        <v>144</v>
+      </c>
+      <c r="C36">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3">
+      <c r="A37" t="s">
+        <v>150</v>
+      </c>
+      <c r="B37" t="s">
+        <v>152</v>
+      </c>
+      <c r="C37">
+        <v>7000</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3">
+      <c r="A38" t="s">
+        <v>157</v>
+      </c>
+      <c r="B38" t="s">
+        <v>159</v>
+      </c>
+      <c r="C38">
+        <v>14000</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3">
+      <c r="A39" t="s">
+        <v>162</v>
+      </c>
+      <c r="B39" t="s">
+        <v>164</v>
+      </c>
+      <c r="C39">
+        <v>770</v>
+      </c>
+    </row>
+    <row r="40" spans="1:3">
+      <c r="A40" t="s">
+        <v>169</v>
+      </c>
+      <c r="B40" t="s">
+        <v>171</v>
+      </c>
+      <c r="C40">
+        <v>560</v>
+      </c>
+    </row>
+    <row r="41" spans="1:3">
+      <c r="A41" t="s">
+        <v>173</v>
+      </c>
+      <c r="B41" t="s">
+        <v>175</v>
+      </c>
+      <c r="C41">
+        <v>560</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{91C92C4B-FFF2-41AF-9776-1DD9E5E0EC98}">
   <sheetPr codeName="Planilha7">
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -3946,577 +4442,577 @@
   <sheetData>
     <row r="1" spans="1:4">
       <c r="A1" s="6" t="s">
+        <v>363</v>
+      </c>
+      <c r="B1" s="6" t="s">
         <v>176</v>
       </c>
-      <c r="B1" s="6" t="s">
+      <c r="C1" s="6" t="s">
         <v>177</v>
-      </c>
-      <c r="C1" s="6" t="s">
-        <v>178</v>
       </c>
       <c r="D1" s="7"/>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="9" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B2" s="8" t="s">
+        <v>229</v>
+      </c>
+      <c r="C2" s="8" t="s">
         <v>230</v>
-      </c>
-      <c r="C2" s="8" t="s">
-        <v>231</v>
       </c>
       <c r="D2" s="7"/>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="9" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B3" s="8" t="s">
+        <v>231</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>232</v>
-      </c>
-      <c r="C3" s="8" t="s">
-        <v>233</v>
       </c>
       <c r="D3" s="7"/>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="9" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B4" s="8" t="s">
+        <v>233</v>
+      </c>
+      <c r="C4" s="8" t="s">
         <v>234</v>
-      </c>
-      <c r="C4" s="8" t="s">
-        <v>235</v>
       </c>
       <c r="D4" s="7"/>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="8" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B5" s="8" t="s">
+        <v>235</v>
+      </c>
+      <c r="C5" s="8" t="s">
         <v>236</v>
-      </c>
-      <c r="C5" s="8" t="s">
-        <v>237</v>
       </c>
       <c r="D5" s="7"/>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="8" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B6" s="8" t="s">
+        <v>237</v>
+      </c>
+      <c r="C6" s="8" t="s">
         <v>238</v>
-      </c>
-      <c r="C6" s="8" t="s">
-        <v>239</v>
       </c>
       <c r="D6" s="7"/>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="8" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B7" s="8" t="s">
+        <v>239</v>
+      </c>
+      <c r="C7" s="8" t="s">
         <v>240</v>
-      </c>
-      <c r="C7" s="8" t="s">
-        <v>241</v>
       </c>
       <c r="D7" s="7"/>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B8" s="8" t="s">
+        <v>241</v>
+      </c>
+      <c r="C8" s="8" t="s">
         <v>242</v>
-      </c>
-      <c r="C8" s="8" t="s">
-        <v>243</v>
       </c>
       <c r="D8" s="7"/>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="8" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B9" s="8" t="s">
+        <v>243</v>
+      </c>
+      <c r="C9" s="8" t="s">
         <v>244</v>
-      </c>
-      <c r="C9" s="8" t="s">
-        <v>245</v>
       </c>
       <c r="D9" s="7"/>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="8" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B10" s="8" t="s">
+        <v>245</v>
+      </c>
+      <c r="C10" s="8" t="s">
         <v>246</v>
-      </c>
-      <c r="C10" s="8" t="s">
-        <v>247</v>
       </c>
       <c r="D10" s="7"/>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="8" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B11" s="8" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="8" t="s">
         <v>248</v>
-      </c>
-      <c r="C11" s="8" t="s">
-        <v>249</v>
       </c>
       <c r="D11" s="7"/>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="8" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B12" s="8" t="s">
+        <v>249</v>
+      </c>
+      <c r="C12" s="8" t="s">
         <v>250</v>
-      </c>
-      <c r="C12" s="8" t="s">
-        <v>251</v>
       </c>
       <c r="D12" s="7"/>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="8" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B13" s="8" t="s">
+        <v>251</v>
+      </c>
+      <c r="C13" s="8" t="s">
         <v>252</v>
-      </c>
-      <c r="C13" s="8" t="s">
-        <v>253</v>
       </c>
       <c r="D13" s="7"/>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="8" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B14" s="8" t="s">
+        <v>253</v>
+      </c>
+      <c r="C14" s="8" t="s">
         <v>254</v>
-      </c>
-      <c r="C14" s="8" t="s">
-        <v>255</v>
       </c>
       <c r="D14" s="7"/>
     </row>
     <row r="15" spans="1:4">
       <c r="A15" s="8" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B15" s="8" t="s">
+        <v>255</v>
+      </c>
+      <c r="C15" s="8" t="s">
         <v>256</v>
-      </c>
-      <c r="C15" s="8" t="s">
-        <v>257</v>
       </c>
       <c r="D15" s="7"/>
     </row>
     <row r="16" spans="1:4">
       <c r="A16" s="8" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B16" s="8" t="s">
+        <v>257</v>
+      </c>
+      <c r="C16" s="8" t="s">
         <v>258</v>
-      </c>
-      <c r="C16" s="8" t="s">
-        <v>259</v>
       </c>
       <c r="D16" s="7"/>
     </row>
     <row r="17" spans="1:4">
       <c r="A17" s="8" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B17" s="8" t="s">
+        <v>259</v>
+      </c>
+      <c r="C17" s="8" t="s">
         <v>260</v>
-      </c>
-      <c r="C17" s="8" t="s">
-        <v>261</v>
       </c>
       <c r="D17" s="7"/>
     </row>
     <row r="18" spans="1:4">
       <c r="A18" s="8" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B18" s="8" t="s">
+        <v>261</v>
+      </c>
+      <c r="C18" s="8" t="s">
         <v>262</v>
-      </c>
-      <c r="C18" s="8" t="s">
-        <v>263</v>
       </c>
       <c r="D18" s="7"/>
     </row>
     <row r="19" spans="1:4">
       <c r="A19" s="8" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B19" s="8" t="s">
+        <v>263</v>
+      </c>
+      <c r="C19" s="8" t="s">
         <v>264</v>
-      </c>
-      <c r="C19" s="8" t="s">
-        <v>265</v>
       </c>
       <c r="D19" s="7"/>
     </row>
     <row r="20" spans="1:4">
       <c r="A20" s="8" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B20" s="8" t="s">
+        <v>265</v>
+      </c>
+      <c r="C20" s="8" t="s">
         <v>266</v>
-      </c>
-      <c r="C20" s="8" t="s">
-        <v>267</v>
       </c>
       <c r="D20" s="7"/>
     </row>
     <row r="21" spans="1:4">
       <c r="A21" s="8" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B21" s="8" t="s">
+        <v>267</v>
+      </c>
+      <c r="C21" s="8" t="s">
         <v>268</v>
-      </c>
-      <c r="C21" s="8" t="s">
-        <v>269</v>
       </c>
       <c r="D21" s="7"/>
     </row>
     <row r="22" spans="1:4">
       <c r="A22" s="8" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B22" s="8" t="s">
+        <v>269</v>
+      </c>
+      <c r="C22" s="8" t="s">
         <v>270</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>271</v>
       </c>
       <c r="D22" s="7"/>
     </row>
     <row r="23" spans="1:4">
       <c r="A23" s="8" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B23" s="8" t="s">
+        <v>271</v>
+      </c>
+      <c r="C23" s="8" t="s">
         <v>272</v>
-      </c>
-      <c r="C23" s="8" t="s">
-        <v>273</v>
       </c>
       <c r="D23" s="7"/>
     </row>
     <row r="24" spans="1:4">
       <c r="A24" s="8" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B24" s="8" t="s">
+        <v>273</v>
+      </c>
+      <c r="C24" s="8" t="s">
         <v>274</v>
-      </c>
-      <c r="C24" s="8" t="s">
-        <v>275</v>
       </c>
       <c r="D24" s="7"/>
     </row>
     <row r="25" spans="1:4">
       <c r="A25" s="8" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B25" s="8" t="s">
+        <v>275</v>
+      </c>
+      <c r="C25" s="8" t="s">
         <v>276</v>
-      </c>
-      <c r="C25" s="8" t="s">
-        <v>277</v>
       </c>
       <c r="D25" s="7"/>
     </row>
     <row r="26" spans="1:4">
       <c r="A26" s="8" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B26" s="8" t="s">
+        <v>277</v>
+      </c>
+      <c r="C26" s="8" t="s">
         <v>278</v>
-      </c>
-      <c r="C26" s="8" t="s">
-        <v>279</v>
       </c>
       <c r="D26" s="7"/>
     </row>
     <row r="27" spans="1:4">
       <c r="A27" s="8" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B27" s="8" t="s">
+        <v>279</v>
+      </c>
+      <c r="C27" s="8" t="s">
         <v>280</v>
-      </c>
-      <c r="C27" s="8" t="s">
-        <v>281</v>
       </c>
       <c r="D27" s="7"/>
     </row>
     <row r="28" spans="1:4">
       <c r="A28" s="8" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B28" s="8" t="s">
+        <v>281</v>
+      </c>
+      <c r="C28" s="8" t="s">
         <v>282</v>
-      </c>
-      <c r="C28" s="8" t="s">
-        <v>283</v>
       </c>
       <c r="D28" s="7"/>
     </row>
     <row r="29" spans="1:4">
       <c r="A29" s="8" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B29" s="8" t="s">
+        <v>283</v>
+      </c>
+      <c r="C29" s="8" t="s">
         <v>284</v>
-      </c>
-      <c r="C29" s="8" t="s">
-        <v>285</v>
       </c>
       <c r="D29" s="7"/>
     </row>
     <row r="30" spans="1:4">
       <c r="A30" s="8" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B30" s="8" t="s">
+        <v>285</v>
+      </c>
+      <c r="C30" s="8" t="s">
         <v>286</v>
-      </c>
-      <c r="C30" s="8" t="s">
-        <v>287</v>
       </c>
       <c r="D30" s="7"/>
     </row>
     <row r="31" spans="1:4">
       <c r="A31" s="8" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B31" s="8" t="s">
+        <v>287</v>
+      </c>
+      <c r="C31" s="8" t="s">
         <v>288</v>
-      </c>
-      <c r="C31" s="8" t="s">
-        <v>289</v>
       </c>
       <c r="D31" s="7"/>
     </row>
     <row r="32" spans="1:4">
       <c r="A32" s="8" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B32" s="8" t="s">
+        <v>289</v>
+      </c>
+      <c r="C32" s="8" t="s">
         <v>290</v>
-      </c>
-      <c r="C32" s="8" t="s">
-        <v>291</v>
       </c>
       <c r="D32" s="7"/>
     </row>
     <row r="33" spans="1:4">
       <c r="A33" s="8" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B33" s="8" t="s">
+        <v>291</v>
+      </c>
+      <c r="C33" s="8" t="s">
         <v>292</v>
-      </c>
-      <c r="C33" s="8" t="s">
-        <v>293</v>
       </c>
       <c r="D33" s="7"/>
     </row>
     <row r="34" spans="1:4">
       <c r="A34" s="8" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B34" s="8" t="s">
+        <v>293</v>
+      </c>
+      <c r="C34" s="8" t="s">
         <v>294</v>
-      </c>
-      <c r="C34" s="8" t="s">
-        <v>295</v>
       </c>
       <c r="D34" s="7"/>
     </row>
     <row r="35" spans="1:4">
       <c r="A35" s="8" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B35" s="8" t="s">
+        <v>295</v>
+      </c>
+      <c r="C35" s="8" t="s">
         <v>296</v>
-      </c>
-      <c r="C35" s="8" t="s">
-        <v>297</v>
       </c>
       <c r="D35" s="7"/>
     </row>
     <row r="36" spans="1:4">
       <c r="A36" s="8" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B36" s="8" t="s">
+        <v>297</v>
+      </c>
+      <c r="C36" s="8" t="s">
         <v>298</v>
-      </c>
-      <c r="C36" s="8" t="s">
-        <v>299</v>
       </c>
       <c r="D36" s="7"/>
     </row>
     <row r="37" spans="1:4">
       <c r="A37" s="8" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B37" s="8" t="s">
+        <v>299</v>
+      </c>
+      <c r="C37" s="8" t="s">
         <v>300</v>
-      </c>
-      <c r="C37" s="8" t="s">
-        <v>301</v>
       </c>
       <c r="D37" s="7"/>
     </row>
     <row r="38" spans="1:4">
       <c r="A38" s="8" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B38" s="8" t="s">
+        <v>301</v>
+      </c>
+      <c r="C38" s="8" t="s">
         <v>302</v>
-      </c>
-      <c r="C38" s="8" t="s">
-        <v>303</v>
       </c>
       <c r="D38" s="7"/>
     </row>
     <row r="39" spans="1:4">
       <c r="A39" s="8"/>
       <c r="B39" s="8" t="s">
+        <v>303</v>
+      </c>
+      <c r="C39" s="8" t="s">
         <v>304</v>
-      </c>
-      <c r="C39" s="8" t="s">
-        <v>305</v>
       </c>
       <c r="D39" s="7"/>
     </row>
     <row r="40" spans="1:4">
       <c r="A40" s="8"/>
       <c r="B40" s="8" t="s">
+        <v>305</v>
+      </c>
+      <c r="C40" s="8" t="s">
         <v>306</v>
-      </c>
-      <c r="C40" s="8" t="s">
-        <v>307</v>
       </c>
       <c r="D40" s="7"/>
     </row>
     <row r="41" spans="1:4">
       <c r="A41" s="8"/>
       <c r="B41" s="8" t="s">
+        <v>307</v>
+      </c>
+      <c r="C41" s="8" t="s">
         <v>308</v>
-      </c>
-      <c r="C41" s="8" t="s">
-        <v>309</v>
       </c>
       <c r="D41" s="7"/>
     </row>
     <row r="42" spans="1:4">
       <c r="A42" s="8"/>
       <c r="B42" s="8" t="s">
+        <v>309</v>
+      </c>
+      <c r="C42" s="8" t="s">
         <v>310</v>
-      </c>
-      <c r="C42" s="8" t="s">
-        <v>311</v>
       </c>
       <c r="D42" s="7"/>
     </row>
     <row r="43" spans="1:4">
       <c r="A43" s="8"/>
       <c r="B43" s="8" t="s">
+        <v>311</v>
+      </c>
+      <c r="C43" s="8" t="s">
         <v>312</v>
-      </c>
-      <c r="C43" s="8" t="s">
-        <v>313</v>
       </c>
       <c r="D43" s="7"/>
     </row>
     <row r="44" spans="1:4">
       <c r="A44" s="8"/>
       <c r="B44" s="8" t="s">
+        <v>313</v>
+      </c>
+      <c r="C44" s="8" t="s">
         <v>314</v>
-      </c>
-      <c r="C44" s="8" t="s">
-        <v>315</v>
       </c>
       <c r="D44" s="7"/>
     </row>
     <row r="45" spans="1:4">
       <c r="A45" s="8"/>
       <c r="B45" s="8" t="s">
+        <v>315</v>
+      </c>
+      <c r="C45" s="8" t="s">
         <v>316</v>
-      </c>
-      <c r="C45" s="8" t="s">
-        <v>317</v>
       </c>
       <c r="D45" s="7"/>
     </row>
     <row r="46" spans="1:4">
       <c r="A46" s="8"/>
       <c r="B46" s="8" t="s">
+        <v>317</v>
+      </c>
+      <c r="C46" s="8" t="s">
         <v>318</v>
-      </c>
-      <c r="C46" s="8" t="s">
-        <v>319</v>
       </c>
       <c r="D46" s="7"/>
     </row>
     <row r="47" spans="1:4">
       <c r="A47" s="8"/>
       <c r="B47" s="8" t="s">
+        <v>319</v>
+      </c>
+      <c r="C47" s="8" t="s">
         <v>320</v>
-      </c>
-      <c r="C47" s="8" t="s">
-        <v>321</v>
       </c>
       <c r="D47" s="7"/>
     </row>
     <row r="48" spans="1:4">
       <c r="A48" s="8"/>
       <c r="B48" s="8" t="s">
+        <v>321</v>
+      </c>
+      <c r="C48" s="8" t="s">
         <v>322</v>
-      </c>
-      <c r="C48" s="8" t="s">
-        <v>323</v>
       </c>
       <c r="D48" s="7"/>
     </row>
     <row r="49" spans="1:4">
       <c r="A49" s="8"/>
       <c r="B49" s="8" t="s">
+        <v>323</v>
+      </c>
+      <c r="C49" s="8" t="s">
         <v>324</v>
-      </c>
-      <c r="C49" s="8" t="s">
-        <v>325</v>
       </c>
       <c r="D49" s="7"/>
     </row>
     <row r="50" spans="1:4">
       <c r="A50" s="8"/>
       <c r="B50" s="8" t="s">
+        <v>325</v>
+      </c>
+      <c r="C50" s="8" t="s">
         <v>326</v>
-      </c>
-      <c r="C50" s="8" t="s">
-        <v>327</v>
       </c>
       <c r="D50" s="7"/>
     </row>
@@ -4524,7 +5020,7 @@
       <c r="A51" s="8"/>
       <c r="B51" s="8"/>
       <c r="C51" s="8" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D51" s="7"/>
     </row>
@@ -4532,7 +5028,7 @@
       <c r="A52" s="8"/>
       <c r="B52" s="8"/>
       <c r="C52" s="8" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="D52" s="7"/>
     </row>
@@ -4540,7 +5036,7 @@
       <c r="A53" s="8"/>
       <c r="B53" s="8"/>
       <c r="C53" s="8" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="D53" s="7"/>
     </row>
@@ -4548,7 +5044,7 @@
       <c r="A54" s="8"/>
       <c r="B54" s="8"/>
       <c r="C54" s="8" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="D54" s="7"/>
     </row>
@@ -4556,7 +5052,7 @@
       <c r="A55" s="8"/>
       <c r="B55" s="8"/>
       <c r="C55" s="8" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="D55" s="7"/>
     </row>
@@ -4564,7 +5060,7 @@
       <c r="A56" s="8"/>
       <c r="B56" s="8"/>
       <c r="C56" s="8" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="D56" s="7"/>
     </row>
@@ -4572,7 +5068,7 @@
       <c r="A57" s="8"/>
       <c r="B57" s="8"/>
       <c r="C57" s="8" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="D57" s="7"/>
     </row>
@@ -4580,7 +5076,7 @@
       <c r="A58" s="8"/>
       <c r="B58" s="8"/>
       <c r="C58" s="8" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="D58" s="7"/>
     </row>
@@ -4588,7 +5084,7 @@
       <c r="A59" s="8"/>
       <c r="B59" s="8"/>
       <c r="C59" s="8" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="D59" s="7"/>
     </row>
@@ -4596,7 +5092,7 @@
       <c r="A60" s="8"/>
       <c r="B60" s="8"/>
       <c r="C60" s="8" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D60" s="7"/>
     </row>
@@ -4604,7 +5100,7 @@
       <c r="A61" s="8"/>
       <c r="B61" s="8"/>
       <c r="C61" s="8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D61" s="7"/>
     </row>
@@ -4612,7 +5108,7 @@
       <c r="A62" s="8"/>
       <c r="B62" s="8"/>
       <c r="C62" s="8" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D62" s="7"/>
     </row>
@@ -4620,7 +5116,7 @@
       <c r="A63" s="8"/>
       <c r="B63" s="8"/>
       <c r="C63" s="8" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D63" s="7"/>
     </row>
@@ -4628,7 +5124,7 @@
       <c r="A64" s="8"/>
       <c r="B64" s="8"/>
       <c r="C64" s="8" t="s">
-        <v>341</v>
+        <v>340</v>
       </c>
       <c r="D64" s="7"/>
     </row>
@@ -4636,7 +5132,7 @@
       <c r="A65" s="8"/>
       <c r="B65" s="8"/>
       <c r="C65" s="8" t="s">
-        <v>342</v>
+        <v>341</v>
       </c>
       <c r="D65" s="7"/>
     </row>
@@ -4644,7 +5140,7 @@
       <c r="A66" s="8"/>
       <c r="B66" s="8"/>
       <c r="C66" s="8" t="s">
-        <v>343</v>
+        <v>342</v>
       </c>
       <c r="D66" s="7"/>
     </row>
@@ -4652,7 +5148,7 @@
       <c r="A67" s="8"/>
       <c r="B67" s="8"/>
       <c r="C67" s="8" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
       <c r="D67" s="7"/>
     </row>
@@ -4660,7 +5156,7 @@
       <c r="A68" s="8"/>
       <c r="B68" s="8"/>
       <c r="C68" s="8" t="s">
-        <v>345</v>
+        <v>344</v>
       </c>
       <c r="D68" s="7"/>
     </row>
@@ -4668,7 +5164,7 @@
       <c r="A69" s="8"/>
       <c r="B69" s="8"/>
       <c r="C69" s="8" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
       <c r="D69" s="7"/>
     </row>
@@ -4676,7 +5172,7 @@
       <c r="A70" s="8"/>
       <c r="B70" s="8"/>
       <c r="C70" s="8" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="D70" s="7"/>
     </row>
@@ -4684,7 +5180,7 @@
       <c r="A71" s="8"/>
       <c r="B71" s="8"/>
       <c r="C71" s="8" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="D71" s="7"/>
     </row>
@@ -4692,7 +5188,7 @@
       <c r="A72" s="8"/>
       <c r="B72" s="8"/>
       <c r="C72" s="8" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
       <c r="D72" s="7"/>
     </row>
@@ -4700,7 +5196,7 @@
       <c r="A73" s="8"/>
       <c r="B73" s="8"/>
       <c r="C73" s="8" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="D73" s="7"/>
     </row>
@@ -4708,7 +5204,7 @@
       <c r="A74" s="8"/>
       <c r="B74" s="8"/>
       <c r="C74" s="8" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="D74" s="7"/>
     </row>
@@ -4716,7 +5212,7 @@
       <c r="A75" s="8"/>
       <c r="B75" s="8"/>
       <c r="C75" s="8" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="D75" s="7"/>
     </row>
@@ -4724,7 +5220,7 @@
       <c r="A76" s="8"/>
       <c r="B76" s="8"/>
       <c r="C76" s="8" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="D76" s="7"/>
     </row>
@@ -4732,7 +5228,7 @@
       <c r="A77" s="8"/>
       <c r="B77" s="8"/>
       <c r="C77" s="8" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
       <c r="D77" s="7"/>
     </row>
@@ -4740,7 +5236,7 @@
       <c r="A78" s="8"/>
       <c r="B78" s="8"/>
       <c r="C78" s="8" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
       <c r="D78" s="7"/>
     </row>
@@ -4748,7 +5244,7 @@
       <c r="A79" s="8"/>
       <c r="B79" s="8"/>
       <c r="C79" s="8" t="s">
-        <v>356</v>
+        <v>355</v>
       </c>
       <c r="D79" s="7"/>
     </row>
@@ -4756,7 +5252,7 @@
       <c r="A80" s="8"/>
       <c r="B80" s="8"/>
       <c r="C80" s="8" t="s">
-        <v>357</v>
+        <v>356</v>
       </c>
       <c r="D80" s="7"/>
     </row>
@@ -4764,7 +5260,7 @@
       <c r="A81" s="8"/>
       <c r="B81" s="8"/>
       <c r="C81" s="8" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
       <c r="D81" s="7"/>
     </row>
@@ -4772,7 +5268,7 @@
       <c r="A82" s="8"/>
       <c r="B82" s="8"/>
       <c r="C82" s="8" t="s">
-        <v>359</v>
+        <v>358</v>
       </c>
       <c r="D82" s="7"/>
     </row>
@@ -4780,7 +5276,7 @@
       <c r="A83" s="8"/>
       <c r="B83" s="8"/>
       <c r="C83" s="8" t="s">
-        <v>360</v>
+        <v>359</v>
       </c>
       <c r="D83" s="7"/>
     </row>
@@ -4788,7 +5284,7 @@
       <c r="A84" s="8"/>
       <c r="B84" s="8"/>
       <c r="C84" s="8" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="D84" s="7"/>
     </row>
@@ -10282,7 +10778,1377 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BE8920D3-94FB-4606-BF59-0B056DF8E525}">
+  <dimension ref="A1:B170"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>368</v>
+      </c>
+      <c r="B1" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>367</v>
+      </c>
+      <c r="B2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>367</v>
+      </c>
+      <c r="B3" t="s">
+        <v>194</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>367</v>
+      </c>
+      <c r="B4" t="s">
+        <v>195</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>367</v>
+      </c>
+      <c r="B5" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="6" spans="1:2">
+      <c r="A6" t="s">
+        <v>367</v>
+      </c>
+      <c r="B6" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="7" spans="1:2">
+      <c r="A7" t="s">
+        <v>367</v>
+      </c>
+      <c r="B7" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8" t="s">
+        <v>367</v>
+      </c>
+      <c r="B8" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9" t="s">
+        <v>367</v>
+      </c>
+      <c r="B9" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10" t="s">
+        <v>367</v>
+      </c>
+      <c r="B10" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="11" spans="1:2">
+      <c r="A11" t="s">
+        <v>367</v>
+      </c>
+      <c r="B11" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12" t="s">
+        <v>367</v>
+      </c>
+      <c r="B12" t="s">
+        <v>203</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13" t="s">
+        <v>367</v>
+      </c>
+      <c r="B13" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14" t="s">
+        <v>367</v>
+      </c>
+      <c r="B14" t="s">
+        <v>205</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15" t="s">
+        <v>367</v>
+      </c>
+      <c r="B15" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="16" spans="1:2">
+      <c r="A16" t="s">
+        <v>367</v>
+      </c>
+      <c r="B16" t="s">
+        <v>207</v>
+      </c>
+    </row>
+    <row r="17" spans="1:2">
+      <c r="A17" t="s">
+        <v>367</v>
+      </c>
+      <c r="B17" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="18" spans="1:2">
+      <c r="A18" t="s">
+        <v>367</v>
+      </c>
+      <c r="B18" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="19" spans="1:2">
+      <c r="A19" t="s">
+        <v>367</v>
+      </c>
+      <c r="B19" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="20" spans="1:2">
+      <c r="A20" t="s">
+        <v>367</v>
+      </c>
+      <c r="B20" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:2">
+      <c r="A21" t="s">
+        <v>367</v>
+      </c>
+      <c r="B21" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="22" spans="1:2">
+      <c r="A22" t="s">
+        <v>367</v>
+      </c>
+      <c r="B22" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="23" spans="1:2">
+      <c r="A23" t="s">
+        <v>367</v>
+      </c>
+      <c r="B23" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="24" spans="1:2">
+      <c r="A24" t="s">
+        <v>367</v>
+      </c>
+      <c r="B24" t="s">
+        <v>214</v>
+      </c>
+    </row>
+    <row r="25" spans="1:2">
+      <c r="A25" t="s">
+        <v>367</v>
+      </c>
+      <c r="B25" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="26" spans="1:2">
+      <c r="A26" t="s">
+        <v>367</v>
+      </c>
+      <c r="B26" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="27" spans="1:2">
+      <c r="A27" t="s">
+        <v>367</v>
+      </c>
+      <c r="B27" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="28" spans="1:2">
+      <c r="A28" t="s">
+        <v>367</v>
+      </c>
+      <c r="B28" t="s">
+        <v>218</v>
+      </c>
+    </row>
+    <row r="29" spans="1:2">
+      <c r="A29" t="s">
+        <v>367</v>
+      </c>
+      <c r="B29" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="30" spans="1:2">
+      <c r="A30" t="s">
+        <v>367</v>
+      </c>
+      <c r="B30" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="31" spans="1:2">
+      <c r="A31" t="s">
+        <v>367</v>
+      </c>
+      <c r="B31" t="s">
+        <v>221</v>
+      </c>
+    </row>
+    <row r="32" spans="1:2">
+      <c r="A32" t="s">
+        <v>367</v>
+      </c>
+      <c r="B32" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="33" spans="1:2">
+      <c r="A33" t="s">
+        <v>367</v>
+      </c>
+      <c r="B33" t="s">
+        <v>223</v>
+      </c>
+    </row>
+    <row r="34" spans="1:2">
+      <c r="A34" t="s">
+        <v>367</v>
+      </c>
+      <c r="B34" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="35" spans="1:2">
+      <c r="A35" t="s">
+        <v>367</v>
+      </c>
+      <c r="B35" t="s">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="36" spans="1:2">
+      <c r="A36" t="s">
+        <v>367</v>
+      </c>
+      <c r="B36" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="37" spans="1:2">
+      <c r="A37" t="s">
+        <v>367</v>
+      </c>
+      <c r="B37" t="s">
+        <v>227</v>
+      </c>
+    </row>
+    <row r="38" spans="1:2">
+      <c r="A38" t="s">
+        <v>367</v>
+      </c>
+      <c r="B38" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="39" spans="1:2">
+      <c r="A39" t="s">
+        <v>369</v>
+      </c>
+      <c r="B39" t="s">
+        <v>229</v>
+      </c>
+    </row>
+    <row r="40" spans="1:2">
+      <c r="A40" t="s">
+        <v>369</v>
+      </c>
+      <c r="B40" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="41" spans="1:2">
+      <c r="A41" t="s">
+        <v>369</v>
+      </c>
+      <c r="B41" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="42" spans="1:2">
+      <c r="A42" t="s">
+        <v>369</v>
+      </c>
+      <c r="B42" t="s">
+        <v>235</v>
+      </c>
+    </row>
+    <row r="43" spans="1:2">
+      <c r="A43" t="s">
+        <v>369</v>
+      </c>
+      <c r="B43" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="44" spans="1:2">
+      <c r="A44" t="s">
+        <v>369</v>
+      </c>
+      <c r="B44" t="s">
+        <v>239</v>
+      </c>
+    </row>
+    <row r="45" spans="1:2">
+      <c r="A45" t="s">
+        <v>369</v>
+      </c>
+      <c r="B45" t="s">
+        <v>241</v>
+      </c>
+    </row>
+    <row r="46" spans="1:2">
+      <c r="A46" t="s">
+        <v>369</v>
+      </c>
+      <c r="B46" t="s">
+        <v>243</v>
+      </c>
+    </row>
+    <row r="47" spans="1:2">
+      <c r="A47" t="s">
+        <v>369</v>
+      </c>
+      <c r="B47" t="s">
+        <v>245</v>
+      </c>
+    </row>
+    <row r="48" spans="1:2">
+      <c r="A48" t="s">
+        <v>369</v>
+      </c>
+      <c r="B48" t="s">
+        <v>247</v>
+      </c>
+    </row>
+    <row r="49" spans="1:2">
+      <c r="A49" t="s">
+        <v>369</v>
+      </c>
+      <c r="B49" t="s">
+        <v>249</v>
+      </c>
+    </row>
+    <row r="50" spans="1:2">
+      <c r="A50" t="s">
+        <v>369</v>
+      </c>
+      <c r="B50" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="51" spans="1:2">
+      <c r="A51" t="s">
+        <v>369</v>
+      </c>
+      <c r="B51" t="s">
+        <v>253</v>
+      </c>
+    </row>
+    <row r="52" spans="1:2">
+      <c r="A52" t="s">
+        <v>369</v>
+      </c>
+      <c r="B52" t="s">
+        <v>255</v>
+      </c>
+    </row>
+    <row r="53" spans="1:2">
+      <c r="A53" t="s">
+        <v>369</v>
+      </c>
+      <c r="B53" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="54" spans="1:2">
+      <c r="A54" t="s">
+        <v>369</v>
+      </c>
+      <c r="B54" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="55" spans="1:2">
+      <c r="A55" t="s">
+        <v>369</v>
+      </c>
+      <c r="B55" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="56" spans="1:2">
+      <c r="A56" t="s">
+        <v>369</v>
+      </c>
+      <c r="B56" t="s">
+        <v>263</v>
+      </c>
+    </row>
+    <row r="57" spans="1:2">
+      <c r="A57" t="s">
+        <v>369</v>
+      </c>
+      <c r="B57" t="s">
+        <v>265</v>
+      </c>
+    </row>
+    <row r="58" spans="1:2">
+      <c r="A58" t="s">
+        <v>369</v>
+      </c>
+      <c r="B58" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="59" spans="1:2">
+      <c r="A59" t="s">
+        <v>369</v>
+      </c>
+      <c r="B59" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="60" spans="1:2">
+      <c r="A60" t="s">
+        <v>369</v>
+      </c>
+      <c r="B60" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="61" spans="1:2">
+      <c r="A61" t="s">
+        <v>369</v>
+      </c>
+      <c r="B61" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="62" spans="1:2">
+      <c r="A62" t="s">
+        <v>369</v>
+      </c>
+      <c r="B62" t="s">
+        <v>275</v>
+      </c>
+    </row>
+    <row r="63" spans="1:2">
+      <c r="A63" t="s">
+        <v>369</v>
+      </c>
+      <c r="B63" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="64" spans="1:2">
+      <c r="A64" t="s">
+        <v>369</v>
+      </c>
+      <c r="B64" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="65" spans="1:2">
+      <c r="A65" t="s">
+        <v>369</v>
+      </c>
+      <c r="B65" t="s">
+        <v>281</v>
+      </c>
+    </row>
+    <row r="66" spans="1:2">
+      <c r="A66" t="s">
+        <v>369</v>
+      </c>
+      <c r="B66" t="s">
+        <v>283</v>
+      </c>
+    </row>
+    <row r="67" spans="1:2">
+      <c r="A67" t="s">
+        <v>369</v>
+      </c>
+      <c r="B67" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="68" spans="1:2">
+      <c r="A68" t="s">
+        <v>369</v>
+      </c>
+      <c r="B68" t="s">
+        <v>287</v>
+      </c>
+    </row>
+    <row r="69" spans="1:2">
+      <c r="A69" t="s">
+        <v>369</v>
+      </c>
+      <c r="B69" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="70" spans="1:2">
+      <c r="A70" t="s">
+        <v>369</v>
+      </c>
+      <c r="B70" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="71" spans="1:2">
+      <c r="A71" t="s">
+        <v>369</v>
+      </c>
+      <c r="B71" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="72" spans="1:2">
+      <c r="A72" t="s">
+        <v>369</v>
+      </c>
+      <c r="B72" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="73" spans="1:2">
+      <c r="A73" t="s">
+        <v>369</v>
+      </c>
+      <c r="B73" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="74" spans="1:2">
+      <c r="A74" t="s">
+        <v>369</v>
+      </c>
+      <c r="B74" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="75" spans="1:2">
+      <c r="A75" t="s">
+        <v>369</v>
+      </c>
+      <c r="B75" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="76" spans="1:2">
+      <c r="A76" t="s">
+        <v>369</v>
+      </c>
+      <c r="B76" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="77" spans="1:2">
+      <c r="A77" t="s">
+        <v>369</v>
+      </c>
+      <c r="B77" t="s">
+        <v>305</v>
+      </c>
+    </row>
+    <row r="78" spans="1:2">
+      <c r="A78" t="s">
+        <v>369</v>
+      </c>
+      <c r="B78" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="79" spans="1:2">
+      <c r="A79" t="s">
+        <v>369</v>
+      </c>
+      <c r="B79" t="s">
+        <v>309</v>
+      </c>
+    </row>
+    <row r="80" spans="1:2">
+      <c r="A80" t="s">
+        <v>369</v>
+      </c>
+      <c r="B80" t="s">
+        <v>311</v>
+      </c>
+    </row>
+    <row r="81" spans="1:2">
+      <c r="A81" t="s">
+        <v>369</v>
+      </c>
+      <c r="B81" t="s">
+        <v>313</v>
+      </c>
+    </row>
+    <row r="82" spans="1:2">
+      <c r="A82" t="s">
+        <v>369</v>
+      </c>
+      <c r="B82" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="83" spans="1:2">
+      <c r="A83" t="s">
+        <v>369</v>
+      </c>
+      <c r="B83" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="84" spans="1:2">
+      <c r="A84" t="s">
+        <v>369</v>
+      </c>
+      <c r="B84" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="85" spans="1:2">
+      <c r="A85" t="s">
+        <v>369</v>
+      </c>
+      <c r="B85" t="s">
+        <v>321</v>
+      </c>
+    </row>
+    <row r="86" spans="1:2">
+      <c r="A86" t="s">
+        <v>369</v>
+      </c>
+      <c r="B86" t="s">
+        <v>323</v>
+      </c>
+    </row>
+    <row r="87" spans="1:2">
+      <c r="A87" t="s">
+        <v>369</v>
+      </c>
+      <c r="B87" t="s">
+        <v>325</v>
+      </c>
+    </row>
+    <row r="88" spans="1:2">
+      <c r="A88" t="s">
+        <v>370</v>
+      </c>
+      <c r="B88" t="s">
+        <v>230</v>
+      </c>
+    </row>
+    <row r="89" spans="1:2">
+      <c r="A89" t="s">
+        <v>370</v>
+      </c>
+      <c r="B89" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="90" spans="1:2">
+      <c r="A90" t="s">
+        <v>370</v>
+      </c>
+      <c r="B90" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="91" spans="1:2">
+      <c r="A91" t="s">
+        <v>370</v>
+      </c>
+      <c r="B91" t="s">
+        <v>236</v>
+      </c>
+    </row>
+    <row r="92" spans="1:2">
+      <c r="A92" t="s">
+        <v>370</v>
+      </c>
+      <c r="B92" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="93" spans="1:2">
+      <c r="A93" t="s">
+        <v>370</v>
+      </c>
+      <c r="B93" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="94" spans="1:2">
+      <c r="A94" t="s">
+        <v>370</v>
+      </c>
+      <c r="B94" t="s">
+        <v>242</v>
+      </c>
+    </row>
+    <row r="95" spans="1:2">
+      <c r="A95" t="s">
+        <v>370</v>
+      </c>
+      <c r="B95" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="96" spans="1:2">
+      <c r="A96" t="s">
+        <v>370</v>
+      </c>
+      <c r="B96" t="s">
+        <v>246</v>
+      </c>
+    </row>
+    <row r="97" spans="1:2">
+      <c r="A97" t="s">
+        <v>370</v>
+      </c>
+      <c r="B97" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="98" spans="1:2">
+      <c r="A98" t="s">
+        <v>370</v>
+      </c>
+      <c r="B98" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="99" spans="1:2">
+      <c r="A99" t="s">
+        <v>370</v>
+      </c>
+      <c r="B99" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="100" spans="1:2">
+      <c r="A100" t="s">
+        <v>370</v>
+      </c>
+      <c r="B100" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="101" spans="1:2">
+      <c r="A101" t="s">
+        <v>370</v>
+      </c>
+      <c r="B101" t="s">
+        <v>256</v>
+      </c>
+    </row>
+    <row r="102" spans="1:2">
+      <c r="A102" t="s">
+        <v>370</v>
+      </c>
+      <c r="B102" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="103" spans="1:2">
+      <c r="A103" t="s">
+        <v>370</v>
+      </c>
+      <c r="B103" t="s">
+        <v>260</v>
+      </c>
+    </row>
+    <row r="104" spans="1:2">
+      <c r="A104" t="s">
+        <v>370</v>
+      </c>
+      <c r="B104" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="105" spans="1:2">
+      <c r="A105" t="s">
+        <v>370</v>
+      </c>
+      <c r="B105" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="106" spans="1:2">
+      <c r="A106" t="s">
+        <v>370</v>
+      </c>
+      <c r="B106" t="s">
+        <v>266</v>
+      </c>
+    </row>
+    <row r="107" spans="1:2">
+      <c r="A107" t="s">
+        <v>370</v>
+      </c>
+      <c r="B107" t="s">
+        <v>268</v>
+      </c>
+    </row>
+    <row r="108" spans="1:2">
+      <c r="A108" t="s">
+        <v>370</v>
+      </c>
+      <c r="B108" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="109" spans="1:2">
+      <c r="A109" t="s">
+        <v>370</v>
+      </c>
+      <c r="B109" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="110" spans="1:2">
+      <c r="A110" t="s">
+        <v>370</v>
+      </c>
+      <c r="B110" t="s">
+        <v>274</v>
+      </c>
+    </row>
+    <row r="111" spans="1:2">
+      <c r="A111" t="s">
+        <v>370</v>
+      </c>
+      <c r="B111" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="112" spans="1:2">
+      <c r="A112" t="s">
+        <v>370</v>
+      </c>
+      <c r="B112" t="s">
+        <v>278</v>
+      </c>
+    </row>
+    <row r="113" spans="1:2">
+      <c r="A113" t="s">
+        <v>370</v>
+      </c>
+      <c r="B113" t="s">
+        <v>280</v>
+      </c>
+    </row>
+    <row r="114" spans="1:2">
+      <c r="A114" t="s">
+        <v>370</v>
+      </c>
+      <c r="B114" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="115" spans="1:2">
+      <c r="A115" t="s">
+        <v>370</v>
+      </c>
+      <c r="B115" t="s">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="116" spans="1:2">
+      <c r="A116" t="s">
+        <v>370</v>
+      </c>
+      <c r="B116" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="117" spans="1:2">
+      <c r="A117" t="s">
+        <v>370</v>
+      </c>
+      <c r="B117" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="118" spans="1:2">
+      <c r="A118" t="s">
+        <v>370</v>
+      </c>
+      <c r="B118" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="119" spans="1:2">
+      <c r="A119" t="s">
+        <v>370</v>
+      </c>
+      <c r="B119" t="s">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="120" spans="1:2">
+      <c r="A120" t="s">
+        <v>370</v>
+      </c>
+      <c r="B120" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="121" spans="1:2">
+      <c r="A121" t="s">
+        <v>370</v>
+      </c>
+      <c r="B121" t="s">
+        <v>296</v>
+      </c>
+    </row>
+    <row r="122" spans="1:2">
+      <c r="A122" t="s">
+        <v>370</v>
+      </c>
+      <c r="B122" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="123" spans="1:2">
+      <c r="A123" t="s">
+        <v>370</v>
+      </c>
+      <c r="B123" t="s">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="124" spans="1:2">
+      <c r="A124" t="s">
+        <v>370</v>
+      </c>
+      <c r="B124" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="125" spans="1:2">
+      <c r="A125" t="s">
+        <v>370</v>
+      </c>
+      <c r="B125" t="s">
+        <v>304</v>
+      </c>
+    </row>
+    <row r="126" spans="1:2">
+      <c r="A126" t="s">
+        <v>370</v>
+      </c>
+      <c r="B126" t="s">
+        <v>306</v>
+      </c>
+    </row>
+    <row r="127" spans="1:2">
+      <c r="A127" t="s">
+        <v>370</v>
+      </c>
+      <c r="B127" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="128" spans="1:2">
+      <c r="A128" t="s">
+        <v>370</v>
+      </c>
+      <c r="B128" t="s">
+        <v>310</v>
+      </c>
+    </row>
+    <row r="129" spans="1:2">
+      <c r="A129" t="s">
+        <v>370</v>
+      </c>
+      <c r="B129" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="130" spans="1:2">
+      <c r="A130" t="s">
+        <v>370</v>
+      </c>
+      <c r="B130" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="131" spans="1:2">
+      <c r="A131" t="s">
+        <v>370</v>
+      </c>
+      <c r="B131" t="s">
+        <v>316</v>
+      </c>
+    </row>
+    <row r="132" spans="1:2">
+      <c r="A132" t="s">
+        <v>370</v>
+      </c>
+      <c r="B132" t="s">
+        <v>318</v>
+      </c>
+    </row>
+    <row r="133" spans="1:2">
+      <c r="A133" t="s">
+        <v>370</v>
+      </c>
+      <c r="B133" t="s">
+        <v>320</v>
+      </c>
+    </row>
+    <row r="134" spans="1:2">
+      <c r="A134" t="s">
+        <v>370</v>
+      </c>
+      <c r="B134" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="135" spans="1:2">
+      <c r="A135" t="s">
+        <v>370</v>
+      </c>
+      <c r="B135" t="s">
+        <v>324</v>
+      </c>
+    </row>
+    <row r="136" spans="1:2">
+      <c r="A136" t="s">
+        <v>370</v>
+      </c>
+      <c r="B136" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="137" spans="1:2">
+      <c r="A137" t="s">
+        <v>370</v>
+      </c>
+      <c r="B137" t="s">
+        <v>327</v>
+      </c>
+    </row>
+    <row r="138" spans="1:2">
+      <c r="A138" t="s">
+        <v>370</v>
+      </c>
+      <c r="B138" t="s">
+        <v>328</v>
+      </c>
+    </row>
+    <row r="139" spans="1:2">
+      <c r="A139" t="s">
+        <v>370</v>
+      </c>
+      <c r="B139" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="140" spans="1:2">
+      <c r="A140" t="s">
+        <v>370</v>
+      </c>
+      <c r="B140" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="141" spans="1:2">
+      <c r="A141" t="s">
+        <v>370</v>
+      </c>
+      <c r="B141" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="142" spans="1:2">
+      <c r="A142" t="s">
+        <v>370</v>
+      </c>
+      <c r="B142" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="143" spans="1:2">
+      <c r="A143" t="s">
+        <v>370</v>
+      </c>
+      <c r="B143" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="144" spans="1:2">
+      <c r="A144" t="s">
+        <v>370</v>
+      </c>
+      <c r="B144" t="s">
+        <v>334</v>
+      </c>
+    </row>
+    <row r="145" spans="1:2">
+      <c r="A145" t="s">
+        <v>370</v>
+      </c>
+      <c r="B145" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="146" spans="1:2">
+      <c r="A146" t="s">
+        <v>370</v>
+      </c>
+      <c r="B146" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="147" spans="1:2">
+      <c r="A147" t="s">
+        <v>370</v>
+      </c>
+      <c r="B147" t="s">
+        <v>337</v>
+      </c>
+    </row>
+    <row r="148" spans="1:2">
+      <c r="A148" t="s">
+        <v>370</v>
+      </c>
+      <c r="B148" t="s">
+        <v>338</v>
+      </c>
+    </row>
+    <row r="149" spans="1:2">
+      <c r="A149" t="s">
+        <v>370</v>
+      </c>
+      <c r="B149" t="s">
+        <v>339</v>
+      </c>
+    </row>
+    <row r="150" spans="1:2">
+      <c r="A150" t="s">
+        <v>370</v>
+      </c>
+      <c r="B150" t="s">
+        <v>340</v>
+      </c>
+    </row>
+    <row r="151" spans="1:2">
+      <c r="A151" t="s">
+        <v>370</v>
+      </c>
+      <c r="B151" t="s">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="152" spans="1:2">
+      <c r="A152" t="s">
+        <v>370</v>
+      </c>
+      <c r="B152" t="s">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="153" spans="1:2">
+      <c r="A153" t="s">
+        <v>370</v>
+      </c>
+      <c r="B153" t="s">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="154" spans="1:2">
+      <c r="A154" t="s">
+        <v>370</v>
+      </c>
+      <c r="B154" t="s">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="155" spans="1:2">
+      <c r="A155" t="s">
+        <v>370</v>
+      </c>
+      <c r="B155" t="s">
+        <v>345</v>
+      </c>
+    </row>
+    <row r="156" spans="1:2">
+      <c r="A156" t="s">
+        <v>370</v>
+      </c>
+      <c r="B156" t="s">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="157" spans="1:2">
+      <c r="A157" t="s">
+        <v>370</v>
+      </c>
+      <c r="B157" t="s">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="158" spans="1:2">
+      <c r="A158" t="s">
+        <v>370</v>
+      </c>
+      <c r="B158" t="s">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="159" spans="1:2">
+      <c r="A159" t="s">
+        <v>370</v>
+      </c>
+      <c r="B159" t="s">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="160" spans="1:2">
+      <c r="A160" t="s">
+        <v>370</v>
+      </c>
+      <c r="B160" t="s">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="161" spans="1:2">
+      <c r="A161" t="s">
+        <v>370</v>
+      </c>
+      <c r="B161" t="s">
+        <v>351</v>
+      </c>
+    </row>
+    <row r="162" spans="1:2">
+      <c r="A162" t="s">
+        <v>370</v>
+      </c>
+      <c r="B162" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="163" spans="1:2">
+      <c r="A163" t="s">
+        <v>370</v>
+      </c>
+      <c r="B163" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="164" spans="1:2">
+      <c r="A164" t="s">
+        <v>370</v>
+      </c>
+      <c r="B164" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="165" spans="1:2">
+      <c r="A165" t="s">
+        <v>370</v>
+      </c>
+      <c r="B165" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="166" spans="1:2">
+      <c r="A166" t="s">
+        <v>370</v>
+      </c>
+      <c r="B166" t="s">
+        <v>356</v>
+      </c>
+    </row>
+    <row r="167" spans="1:2">
+      <c r="A167" t="s">
+        <v>370</v>
+      </c>
+      <c r="B167" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="168" spans="1:2">
+      <c r="A168" t="s">
+        <v>370</v>
+      </c>
+      <c r="B168" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="169" spans="1:2">
+      <c r="A169" t="s">
+        <v>370</v>
+      </c>
+      <c r="B169" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="170" spans="1:2">
+      <c r="A170" t="s">
+        <v>370</v>
+      </c>
+      <c r="B170" t="s">
+        <v>360</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4D39724D-3F66-41F4-94FA-CB4D74AA64A8}">
   <sheetPr codeName="Planilha8">
     <outlinePr summaryBelow="0" summaryRight="0"/>
@@ -10298,10 +12164,10 @@
   <sheetData>
     <row r="1" spans="1:24">
       <c r="A1" s="16" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B1" s="17" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="C1" s="5"/>
       <c r="D1" s="5"/>
@@ -10328,7 +12194,7 @@
     </row>
     <row r="2" spans="1:24" ht="45">
       <c r="A2" s="18" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B2" s="19">
         <v>425</v>
@@ -10358,7 +12224,7 @@
     </row>
     <row r="3" spans="1:24" ht="30">
       <c r="A3" s="18" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B3" s="19">
         <v>380</v>
@@ -10388,7 +12254,7 @@
     </row>
     <row r="4" spans="1:24">
       <c r="A4" s="20" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B4" s="21">
         <v>335</v>
@@ -10418,7 +12284,7 @@
     </row>
     <row r="5" spans="1:24" ht="15.75" thickBot="1">
       <c r="A5" s="22" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B5" s="23">
         <f>370*5.5</f>
@@ -35985,7 +37851,112 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8DB018A6-B7E7-4ACD-B818-12EC82A1C9F4}">
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:2">
+      <c r="A1" t="s">
+        <v>371</v>
+      </c>
+      <c r="B1" t="s">
+        <v>372</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
+      <c r="A2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B2">
+        <v>425</v>
+      </c>
+    </row>
+    <row r="3" spans="1:2">
+      <c r="A3" t="s">
+        <v>181</v>
+      </c>
+      <c r="B3">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
+      <c r="A4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B4">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
+      <c r="A5" t="s">
+        <v>183</v>
+      </c>
+      <c r="B5">
+        <v>2035</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{DAA83A0C-D0FE-4BDC-8F1C-42DE6CCF5084}">
+  <dimension ref="A1:A9"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="2" spans="1:1">
+      <c r="A2" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1">
+      <c r="A3" t="s">
+        <v>186</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1">
+      <c r="A4" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:1">
+      <c r="A5" t="s">
+        <v>188</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1">
+      <c r="A6" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="7" spans="1:1">
+      <c r="A7" t="s">
+        <v>190</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1">
+      <c r="A8" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="9" spans="1:1">
+      <c r="A9" t="s">
+        <v>192</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4C384FF0-2BF5-4867-9EF7-EAAFC6C483C3}">
   <sheetPr codeName="Planilha10"/>
   <dimension ref="A1:A15"/>
@@ -35996,47 +37967,47 @@
   <sheetData>
     <row r="1" spans="1:1" ht="19.5" thickBot="1">
       <c r="A1" s="12" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
     </row>
     <row r="2" spans="1:1">
       <c r="A2" s="13" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" spans="1:1">
       <c r="A3" s="13" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
     </row>
     <row r="4" spans="1:1">
       <c r="A4" s="13" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
     </row>
     <row r="5" spans="1:1">
       <c r="A5" s="13" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
     </row>
     <row r="6" spans="1:1">
       <c r="A6" s="13" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
     </row>
     <row r="7" spans="1:1">
       <c r="A7" s="13" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
     </row>
     <row r="8" spans="1:1">
       <c r="A8" s="13" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="9" spans="1:1" ht="15.75" thickBot="1">
       <c r="A9" s="14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="10" spans="1:1">

</xml_diff>